<commit_message>
Tarif: sommersatser bruges (ét sæt perioder, to sæt satser)
</commit_message>
<xml_diff>
--- a/doc/vaerksdata_skabelon.xlsx
+++ b/doc/vaerksdata_skabelon.xlsx
@@ -440,7 +440,7 @@
     <t xml:space="preserve">Tidsvarierende nettarif</t>
   </si>
   <si>
-    <t xml:space="preserve">De tre bånd står på dit netselskabs prisblad, typisk som lavlast, højlast og spidslast. Har dit selskab andre navne eller flere bånd, så skriv dem, du har — resten kan stå tomme. Tidspunkterne er faste i modellen og følger inddelingen i noterne til højre. Bruger jeres netselskab andre tidspunkter — fx spidslast kl. 17–21 — så skriv jeres tidspunkter i mailen, når du sender arket.</t>
+    <t xml:space="preserve">De tre bånd står på dit netselskabs prisblad, typisk som lavlast, højlast og spidslast. Har dit selskab andre navne eller flere bånd, så skriv dem, du har — resten kan stå tomme. Er satserne forskellige vinter og sommer, så udfyld begge kolonner. Tidspunkterne er faste i modellen og følger inddelingen i noterne til højre. Bruger jeres netselskab andre tidspunkter — fx spidslast kl. 17–21 — så skriv jeres tidspunkter i mailen, når du sender arket.</t>
   </si>
   <si>
     <t xml:space="preserve">bånd</t>
@@ -2709,7 +2709,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="25" t="s">
         <v>138</v>
       </c>

</xml_diff>